<commit_message>
feat: implement product automation and price checker; ignore large data files and tokens
</commit_message>
<xml_diff>
--- a/Recorded/hurtownie_allegro.xlsx
+++ b/Recorded/hurtownie_allegro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bedna\Documents\Robocorp\Gapli\Recorded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64A6FB1-5E36-449F-AE0A-11763DA4DDB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D527C0E0-E0A8-473C-9436-FE4F7BD9CB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hurtownie Allegro" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="177">
   <si>
     <t>Nazwa Hurtowni</t>
   </si>
@@ -97,9 +97,6 @@
     <t>BIO Planet</t>
   </si>
   <si>
-    <t>BOSSOFTOYS</t>
-  </si>
-  <si>
     <t>Brits</t>
   </si>
   <si>
@@ -139,9 +136,6 @@
     <t>🟡 59</t>
   </si>
   <si>
-    <t>Dkaren</t>
-  </si>
-  <si>
     <t>Dla domu i ogrodu</t>
   </si>
   <si>
@@ -211,9 +205,6 @@
     <t>FreeForm</t>
   </si>
   <si>
-    <t>FToys</t>
-  </si>
-  <si>
     <t>Galanter</t>
   </si>
   <si>
@@ -560,9 +551,6 @@
   </si>
   <si>
     <t>WEGA</t>
-  </si>
-  <si>
-    <t>Wyprzedaż Gapli</t>
   </si>
 </sst>
 </file>
@@ -902,10 +890,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C158"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C154"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -916,7 +907,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -924,7 +915,7 @@
         <v>8395</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -932,7 +923,7 @@
         <v>1936</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -943,7 +934,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -954,7 +945,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -962,7 +953,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -970,7 +961,7 @@
         <v>8036</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -978,7 +969,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -989,7 +980,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -997,7 +988,7 @@
         <v>2954</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1005,7 +996,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1013,7 +1004,7 @@
         <v>1170</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1021,7 +1012,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1032,7 +1023,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1040,7 +1031,7 @@
         <v>3305</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1048,7 +1039,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1056,7 +1047,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1064,7 +1055,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1072,1188 +1063,1153 @@
         <v>4947</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
       <c r="B20">
-        <v>17029</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16846</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>26</v>
       </c>
       <c r="B21">
-        <v>16846</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>27</v>
       </c>
       <c r="B22">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>28</v>
       </c>
       <c r="B23">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>29</v>
       </c>
       <c r="B24">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>30</v>
       </c>
       <c r="B25">
-        <v>1263</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>31</v>
       </c>
       <c r="B26">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>32</v>
       </c>
       <c r="B27">
-        <v>1703</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+        <v>16833</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>33</v>
       </c>
       <c r="B28">
-        <v>16833</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
       <c r="B29">
-        <v>762</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1523</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>35</v>
       </c>
       <c r="B30">
-        <v>1523</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>36</v>
       </c>
       <c r="B31">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1164</v>
+      </c>
+      <c r="C31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B32">
-        <v>1164</v>
-      </c>
-      <c r="C32" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4613</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>39</v>
       </c>
       <c r="B33">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>40</v>
       </c>
       <c r="B34">
-        <v>4613</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>41</v>
       </c>
       <c r="B35">
-        <v>1274</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>42</v>
       </c>
       <c r="B36">
-        <v>2930</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2866</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>43</v>
       </c>
       <c r="B37">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+        <v>23199</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>44</v>
       </c>
       <c r="B38">
-        <v>2866</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3323</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>45</v>
       </c>
       <c r="B39">
-        <v>23199</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>46</v>
       </c>
       <c r="B40">
-        <v>3323</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>47</v>
       </c>
       <c r="B41">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1236</v>
+      </c>
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B42">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B43">
-        <v>1236</v>
+        <v>1503</v>
       </c>
       <c r="C43" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B44">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10990</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B45">
-        <v>1503</v>
-      </c>
-      <c r="C45" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+        <v>13991</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>54</v>
       </c>
       <c r="B46">
-        <v>10990</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>55</v>
       </c>
       <c r="B47">
-        <v>13991</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+        <v>918</v>
+      </c>
+      <c r="C47" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B48">
-        <v>1128</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B49">
-        <v>918</v>
-      </c>
-      <c r="C49" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>59</v>
       </c>
       <c r="B50">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6248</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>60</v>
       </c>
       <c r="B51">
-        <v>2046</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2367</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>61</v>
       </c>
       <c r="B52">
-        <v>6248</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2368</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>62</v>
       </c>
       <c r="B53">
-        <v>2367</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>63</v>
       </c>
       <c r="B54">
-        <v>1456</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>64</v>
       </c>
       <c r="B55">
-        <v>2368</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6182</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>65</v>
       </c>
       <c r="B56">
-        <v>2416</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1420</v>
+      </c>
+      <c r="C56" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B57">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6473</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B58">
-        <v>6182</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6056</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B59">
-        <v>1420</v>
-      </c>
-      <c r="C59" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>70</v>
       </c>
       <c r="B60">
-        <v>6473</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>71</v>
       </c>
       <c r="B61">
-        <v>6056</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>72</v>
       </c>
       <c r="B62">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21929</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>73</v>
       </c>
       <c r="B63">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>74</v>
       </c>
       <c r="B64">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>75</v>
       </c>
       <c r="B65">
-        <v>21929</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>76</v>
       </c>
       <c r="B66">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>77</v>
       </c>
       <c r="B67">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8461</v>
+      </c>
+      <c r="C67" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B68">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B69">
-        <v>1543</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+        <v>12590</v>
+      </c>
+      <c r="C69" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B70">
-        <v>8461</v>
-      </c>
-      <c r="C70" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B71">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2572</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B72">
-        <v>12590</v>
-      </c>
-      <c r="C72" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>85</v>
       </c>
       <c r="B73">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>86</v>
       </c>
       <c r="B74">
-        <v>2572</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2566</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>87</v>
       </c>
       <c r="B75">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2587</v>
+      </c>
+      <c r="C75" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>89</v>
+      </c>
+      <c r="B76">
+        <v>5321</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>90</v>
+      </c>
+      <c r="B77">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>91</v>
+      </c>
+      <c r="B78">
+        <v>9605</v>
+      </c>
+      <c r="C78" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>93</v>
+      </c>
+      <c r="B79">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>94</v>
+      </c>
+      <c r="B80">
+        <v>14543</v>
+      </c>
+      <c r="C80" t="s">
         <v>88</v>
       </c>
-      <c r="B76">
-        <v>722</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>89</v>
-      </c>
-      <c r="B77">
-        <v>2566</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>90</v>
-      </c>
-      <c r="B78">
-        <v>2587</v>
-      </c>
-      <c r="C78" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>92</v>
-      </c>
-      <c r="B79">
-        <v>5321</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>93</v>
-      </c>
-      <c r="B80">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B81">
-        <v>9605</v>
-      </c>
-      <c r="C81" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1753</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>96</v>
       </c>
       <c r="B82">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2598</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>97</v>
       </c>
       <c r="B83">
-        <v>14543</v>
+        <v>1243</v>
       </c>
       <c r="C83" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>98</v>
       </c>
       <c r="B84">
-        <v>1753</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2231</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>99</v>
       </c>
       <c r="B85">
-        <v>2598</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9588</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>100</v>
       </c>
       <c r="B86">
-        <v>1243</v>
-      </c>
-      <c r="C86" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+        <v>7564</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>101</v>
       </c>
       <c r="B87">
-        <v>2231</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1618</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>102</v>
       </c>
       <c r="B88">
-        <v>9588</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2134</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>103</v>
       </c>
       <c r="B89">
-        <v>7564</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>104</v>
       </c>
       <c r="B90">
-        <v>1618</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>105</v>
       </c>
       <c r="B91">
-        <v>2134</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>106</v>
       </c>
       <c r="B92">
-        <v>1692</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>107</v>
       </c>
       <c r="B93">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8970</v>
+      </c>
+      <c r="C93" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>108</v>
       </c>
       <c r="B94">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>109</v>
       </c>
       <c r="B95">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6213</v>
+      </c>
+      <c r="C95" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>110</v>
       </c>
       <c r="B96">
-        <v>8970</v>
-      </c>
-      <c r="C96" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+        <v>5702</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>111</v>
       </c>
       <c r="B97">
-        <v>1021</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+        <v>30245</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>112</v>
       </c>
       <c r="B98">
-        <v>6213</v>
-      </c>
-      <c r="C98" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>113</v>
       </c>
       <c r="B99">
-        <v>5702</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2756</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>114</v>
       </c>
       <c r="B100">
-        <v>30245</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>115</v>
       </c>
       <c r="B101">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6466</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>116</v>
       </c>
       <c r="B102">
-        <v>2756</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3986</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>117</v>
       </c>
       <c r="B103">
-        <v>1074</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+        <v>920</v>
+      </c>
+      <c r="C103" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B104">
-        <v>6466</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+        <v>25969</v>
+      </c>
+      <c r="C104" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B105">
-        <v>3986</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3640</v>
+      </c>
+      <c r="C105" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B106">
-        <v>920</v>
+        <v>111299</v>
       </c>
       <c r="C106" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B107">
-        <v>25969</v>
-      </c>
-      <c r="C107" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B108">
-        <v>3640</v>
-      </c>
-      <c r="C108" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B109">
-        <v>111299</v>
-      </c>
-      <c r="C109" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>128</v>
       </c>
       <c r="B110">
-        <v>1192</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>129</v>
       </c>
       <c r="B111">
-        <v>2496</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>130</v>
       </c>
       <c r="B112">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>131</v>
       </c>
       <c r="B113">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+        <v>409</v>
+      </c>
+      <c r="C113" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B114">
-        <v>1175</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2534</v>
+      </c>
+      <c r="C114" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B115">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B116">
-        <v>409</v>
+        <v>2838</v>
       </c>
       <c r="C116" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B117">
-        <v>2534</v>
-      </c>
-      <c r="C117" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>138</v>
       </c>
       <c r="B118">
-        <v>1537</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8655</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>139</v>
       </c>
       <c r="B119">
-        <v>2838</v>
-      </c>
-      <c r="C119" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>140</v>
       </c>
       <c r="B120">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>141</v>
       </c>
       <c r="B121">
-        <v>8655</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>142</v>
       </c>
       <c r="B122">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>143</v>
       </c>
       <c r="B123">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1798</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>144</v>
       </c>
       <c r="B124">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1544</v>
+      </c>
+      <c r="C124" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>145</v>
       </c>
       <c r="B125">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4719</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>146</v>
       </c>
       <c r="B126">
-        <v>1798</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>147</v>
       </c>
       <c r="B127">
-        <v>1544</v>
-      </c>
-      <c r="C127" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>148</v>
       </c>
       <c r="B128">
-        <v>4719</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>149</v>
       </c>
       <c r="B129">
-        <v>1385</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>150</v>
       </c>
       <c r="B130">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+        <v>11755</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>151</v>
       </c>
       <c r="B131">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>152</v>
       </c>
       <c r="B132">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>153</v>
       </c>
       <c r="B133">
-        <v>11755</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>154</v>
       </c>
       <c r="B134">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2336</v>
+      </c>
+      <c r="C134" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B135">
-        <v>1463</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8091</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B136">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+      <c r="C136" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B137">
-        <v>2336</v>
-      </c>
-      <c r="C137" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B138">
-        <v>8091</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B139">
-        <v>290</v>
-      </c>
-      <c r="C139" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+        <v>19595</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>162</v>
       </c>
       <c r="B140">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>163</v>
       </c>
       <c r="B141">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>164</v>
       </c>
       <c r="B142">
-        <v>19595</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>165</v>
       </c>
       <c r="B143">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>166</v>
       </c>
       <c r="B144">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1924</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>167</v>
       </c>
       <c r="B145">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>168</v>
       </c>
       <c r="B146">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>169</v>
       </c>
       <c r="B147">
-        <v>1924</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4615</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>170</v>
       </c>
       <c r="B148">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+        <v>9471</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>171</v>
       </c>
       <c r="B149">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>172</v>
       </c>
       <c r="B150">
-        <v>4615</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>173</v>
       </c>
       <c r="B151">
-        <v>9471</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>174</v>
       </c>
       <c r="B152">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>175</v>
       </c>
       <c r="B153">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3503</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>176</v>
       </c>
       <c r="B154">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A155" t="s">
-        <v>177</v>
-      </c>
-      <c r="B155">
-        <v>1066</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
-        <v>178</v>
-      </c>
-      <c r="B156">
-        <v>3503</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>179</v>
-      </c>
-      <c r="B157">
         <v>38823</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
-        <v>180</v>
-      </c>
-      <c r="B158">
-        <v>446</v>
-      </c>
-      <c r="C158" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>